<commit_message>
CNS: add institutional won-but-unfunded pipeline (KPI, chart, table, CSV/Excel)
</commit_message>
<xml_diff>
--- a/data/company-CNS.xlsx
+++ b/data/company-CNS.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,40 +479,45 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>Won-but-unfunded pipeline</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Organic growth (ann.)*</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Revenue (GAAP)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Revenue (adj.)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Effective fee rate*</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Reported fee rate ex perf.</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Op. margin (as adj.)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Adj. diluted EPS</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -557,29 +562,32 @@
         <v>0.02</v>
       </c>
       <c r="L2" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="M2" t="n">
         <v>7.4</v>
       </c>
-      <c r="M2" t="n">
+      <c r="N2" t="n">
         <v>159.6</v>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>159.7</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>62.9</v>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>51.7</v>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>1.24</v>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481222000036/cns-earningsreleasex123121.htm</t>
         </is>
@@ -624,29 +632,32 @@
         <v>0.55</v>
       </c>
       <c r="L3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M3" t="n">
         <v>2.8</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>154.2</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>154.3</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>61</v>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>44.7</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>1.04</v>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481222000156/cns-earningsreleasex33122e.htm</t>
         </is>
@@ -691,29 +702,32 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="M4" t="n">
         <v>-2.8</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>147.4</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>147.7</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>62.1</v>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>43.3</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>0.96</v>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481222000206/cns-earningsreleasex63022e.htm</t>
         </is>
@@ -758,29 +772,32 @@
         <v>0.01</v>
       </c>
       <c r="L5" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="M5" t="n">
         <v>-2.7</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>140</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>140.2</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>62.5</v>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>42.8</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>0.92</v>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481222000256/cns-earningsreleasex93022e.htm</t>
         </is>
@@ -825,29 +842,32 @@
         <v>0.01</v>
       </c>
       <c r="L6" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="M6" t="n">
         <v>-5.5</v>
       </c>
-      <c r="M6" t="n">
+      <c r="N6" t="n">
         <v>125.3</v>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>125.5</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>62.3</v>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>40.5</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>0.79</v>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481223000018/cns-earningsreleasex123122.htm</t>
         </is>
@@ -892,29 +912,32 @@
         <v>-0.07000000000000001</v>
       </c>
       <c r="L7" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="M7" t="n">
         <v>-2.5</v>
       </c>
-      <c r="M7" t="n">
+      <c r="N7" t="n">
         <v>126.1</v>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>126.3</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>60.7</v>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>38</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>0.76</v>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481223000151/cns-earningsreleasex33123e.htm</t>
         </is>
@@ -959,29 +982,32 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="M8" t="n">
         <v>-2.6</v>
       </c>
-      <c r="M8" t="n">
+      <c r="N8" t="n">
         <v>120.6</v>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>120.3</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>60.6</v>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>36.4</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>0.7</v>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481223000216/cns-earningsreleasex63023e.htm</t>
         </is>
@@ -1026,29 +1052,32 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="M9" t="n">
         <v>-0.2</v>
       </c>
-      <c r="M9" t="n">
+      <c r="N9" t="n">
         <v>123.7</v>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>123.6</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>61.8</v>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>35.5</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>0.7</v>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481223000277/cns-earningsreleasex93023e.htm</t>
         </is>
@@ -1093,29 +1122,32 @@
         <v>-0</v>
       </c>
       <c r="L10" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M10" t="n">
         <v>-5</v>
       </c>
-      <c r="M10" t="n">
+      <c r="N10" t="n">
         <v>119.2</v>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>119</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>61.9</v>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>34.7</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>0.67</v>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481224000020/cns-earningsreleasex123123.htm</t>
         </is>
@@ -1160,29 +1192,32 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
         <v>-9.5</v>
       </c>
-      <c r="M11" t="n">
+      <c r="N11" t="n">
         <v>122.7</v>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>122.9</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>61.3</v>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>35.5</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>0.7</v>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481224000186/cns-earningsreleasex33124e.htm</t>
         </is>
@@ -1227,29 +1262,32 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
         <v>-1.7</v>
       </c>
-      <c r="M12" t="n">
+      <c r="N12" t="n">
         <v>121.7</v>
       </c>
-      <c r="N12" t="n">
+      <c r="O12" t="n">
         <v>122</v>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>61.3</v>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>34.9</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>0.68</v>
       </c>
-      <c r="S12" t="inlineStr">
+      <c r="T12" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481224000267/cns-earningsreleasex63024e.htm</t>
         </is>
@@ -1294,29 +1332,32 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
+        <v>0.651</v>
+      </c>
+      <c r="M13" t="n">
         <v>6.4</v>
       </c>
-      <c r="M13" t="n">
+      <c r="N13" t="n">
         <v>133.2</v>
       </c>
-      <c r="N13" t="n">
+      <c r="O13" t="n">
         <v>133.4</v>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>61.9</v>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>35.7</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>0.77</v>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481224000351/cns-earningsreleasex93024e.htm</t>
         </is>
@@ -1361,29 +1402,32 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
+        <v>0.531</v>
+      </c>
+      <c r="M14" t="n">
         <v>3.7</v>
       </c>
-      <c r="M14" t="n">
+      <c r="N14" t="n">
         <v>139.8</v>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>139.9</v>
       </c>
-      <c r="O14" t="n">
+      <c r="P14" t="n">
         <v>62.6</v>
       </c>
-      <c r="P14" t="inlineStr">
+      <c r="Q14" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q14" t="n">
+      <c r="R14" t="n">
         <v>35.5</v>
       </c>
-      <c r="R14" t="n">
+      <c r="S14" t="n">
         <v>0.78</v>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481225000024/cns-earningsreleasex123124.htm</t>
         </is>
@@ -1428,29 +1472,32 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
+        <v>0.061</v>
+      </c>
+      <c r="M15" t="n">
         <v>1</v>
       </c>
-      <c r="M15" t="n">
+      <c r="N15" t="n">
         <v>134.5</v>
       </c>
-      <c r="N15" t="n">
+      <c r="O15" t="n">
         <v>133.8</v>
       </c>
-      <c r="O15" t="n">
+      <c r="P15" t="n">
         <v>61.7</v>
       </c>
-      <c r="P15" t="inlineStr">
+      <c r="Q15" t="inlineStr">
         <is>
           <t>n/a</t>
         </is>
       </c>
-      <c r="Q15" t="n">
+      <c r="R15" t="n">
         <v>34.7</v>
       </c>
-      <c r="R15" t="n">
+      <c r="S15" t="n">
         <v>0.75</v>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481225000152/cns-earningsreleasex33125e.htm</t>
         </is>
@@ -1495,27 +1542,30 @@
         <v>0.1</v>
       </c>
       <c r="L16" t="n">
+        <v>0.776</v>
+      </c>
+      <c r="M16" t="n">
         <v>-0.6</v>
       </c>
-      <c r="M16" t="n">
+      <c r="N16" t="n">
         <v>136.1</v>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>135.3</v>
       </c>
-      <c r="O16" t="n">
+      <c r="P16" t="n">
         <v>62</v>
       </c>
-      <c r="P16" t="n">
+      <c r="Q16" t="n">
         <v>59.1</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="R16" t="n">
         <v>33.6</v>
       </c>
-      <c r="R16" t="n">
+      <c r="S16" t="n">
         <v>0.73</v>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481225000248/cns-earningsreleasex63025e.htm</t>
         </is>
@@ -1560,27 +1610,30 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="M17" t="n">
         <v>1</v>
       </c>
-      <c r="M17" t="n">
+      <c r="N17" t="n">
         <v>141.7</v>
       </c>
-      <c r="N17" t="n">
+      <c r="O17" t="n">
         <v>140.9</v>
       </c>
-      <c r="O17" t="n">
+      <c r="P17" t="n">
         <v>62.8</v>
       </c>
-      <c r="P17" t="n">
+      <c r="Q17" t="n">
         <v>59.1</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="R17" t="n">
         <v>36.1</v>
       </c>
-      <c r="R17" t="n">
+      <c r="S17" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="S17" t="inlineStr">
+      <c r="T17" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481225000296/cns-earningsreleasex93025e.htm</t>
         </is>
@@ -1625,27 +1678,30 @@
         <v>0.51</v>
       </c>
       <c r="L18" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="M18" t="n">
         <v>5.3</v>
-      </c>
-      <c r="M18" t="n">
-        <v>143.8</v>
       </c>
       <c r="N18" t="n">
         <v>143.8</v>
       </c>
       <c r="O18" t="n">
+        <v>143.8</v>
+      </c>
+      <c r="P18" t="n">
         <v>63.4</v>
       </c>
-      <c r="P18" t="n">
+      <c r="Q18" t="n">
         <v>58.7</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="R18" t="n">
         <v>36.4</v>
       </c>
-      <c r="R18" t="n">
+      <c r="S18" t="n">
         <v>0.8100000000000001</v>
       </c>
-      <c r="S18" t="inlineStr">
+      <c r="T18" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481226000006/cns-earningsreleasex123125.htm</t>
         </is>
@@ -1690,27 +1746,30 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="M19" t="n">
         <v>2.2</v>
       </c>
-      <c r="M19" t="n">
+      <c r="N19" t="n">
         <v>145.6</v>
       </c>
-      <c r="N19" t="n">
+      <c r="O19" t="n">
         <v>144.3</v>
       </c>
-      <c r="O19" t="n">
+      <c r="P19" t="n">
         <v>61.2</v>
       </c>
-      <c r="P19" t="n">
+      <c r="Q19" t="n">
         <v>59</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="R19" t="n">
         <v>35.1</v>
       </c>
-      <c r="R19" t="n">
+      <c r="S19" t="n">
         <v>0.79</v>
       </c>
-      <c r="S19" t="inlineStr">
+      <c r="T19" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481226000035/cns-earningsreleasex33126e.htm</t>
         </is>
@@ -1755,27 +1814,30 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="M20" t="n">
         <v>5.6</v>
       </c>
-      <c r="M20" t="n">
+      <c r="N20" t="n">
         <v>152.7</v>
       </c>
-      <c r="N20" t="n">
+      <c r="O20" t="n">
         <v>151.8</v>
       </c>
-      <c r="O20" t="n">
+      <c r="P20" t="n">
         <v>61.4</v>
       </c>
-      <c r="P20" t="n">
+      <c r="Q20" t="n">
         <v>58.5</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="R20" t="n">
         <v>36.3</v>
       </c>
-      <c r="R20" t="n">
+      <c r="S20" t="n">
         <v>0.85</v>
       </c>
-      <c r="S20" t="inlineStr">
+      <c r="T20" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481226000142/cns-earningsreleasex63026e.htm</t>
         </is>
@@ -1820,27 +1882,30 @@
         <v>0.2</v>
       </c>
       <c r="L21" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="M21" t="n">
         <v>6.2</v>
       </c>
-      <c r="M21" t="n">
+      <c r="N21" t="n">
         <v>157.4</v>
       </c>
-      <c r="N21" t="n">
+      <c r="O21" t="n">
         <v>156.4</v>
       </c>
-      <c r="O21" t="n">
+      <c r="P21" t="n">
         <v>61.9</v>
       </c>
-      <c r="P21" t="n">
+      <c r="Q21" t="n">
         <v>58.3</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="R21" t="n">
         <v>37.2</v>
       </c>
-      <c r="R21" t="n">
+      <c r="S21" t="n">
         <v>0.89</v>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>https://www.sec.gov/Archives/edgar/data/1284812/000128481226000195/cns-earningsreleasex93026e.htm</t>
         </is>
@@ -1857,7 +1922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1884,6 +1949,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Won-but-unfunded pipeline: institutional mandates awarded but not yet funded, $bn at quarter end. Not in the 8-K exhibits (checked all 20 filings); taken from the CEO's prepared remarks on each earnings call (transcript links in companies/raw/cns_pipeline.json). Values are as stated on the call, often rounded (e.g. $1.1bn). Q1 2023, Q1 2024 and Q3 2024 come from the following quarter's call ('compared with $X last quarter').</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>Reported fee rate (ex performance fees) is first disclosed in the Q2 2026 release (with history back to Q2 2025); earlier quarters n/a.</t>
         </is>
       </c>

</xml_diff>